<commit_message>
fix(coffee-shop-checklists-en): ronda 1 de la revisión adversarial — 5 MAYOR + 15 menor aplicados
Leche abierta 7 días (FDA 3-501.17(B)), tiras de sanitizante en tareas diarias, cold brew, hollandaise 135 °F
o 4 h (3-501.19) y aviso al consumidor (3-603.11), restos de restaurante fuera. Gate nuevo TERMINOS_PROHIBIDOS
por kit en G2 (+ autotest 18/18). Base y bar idénticos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Via: Claude Code
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/coffee-shop-checklist-templates/01-coffee-shop-opening-closing-checklists.xlsx
+++ b/astro-site/public/dl/coffee-shop-checklist-templates/01-coffee-shop-opening-closing-checklists.xlsx
@@ -1199,7 +1199,7 @@
       </c>
       <c r="B17" s="28" t="inlineStr">
         <is>
-          <t>Check that the walk-in cooler and freezer ran all night and log the temperature (cooler 41 °F or below, freezer 0 °F or below) — log reading: ____ °F. If out of range, don't use the product until it's been assessed</t>
+          <t>Check that the coolers (walk-in or reach-in) and the freezer ran all night and log the temperatures (cooler 41 °F or below, freezer 0 °F or below) — log reading: cooler ____ °F · freezer ____ °F. If out of range, don't use the product until it's been assessed</t>
         </is>
       </c>
       <c r="C17" s="29" t="inlineStr">
@@ -1372,9 +1372,9 @@
       <c r="A24" s="31" t="n">
         <v>17</v>
       </c>
-      <c r="B24" s="32" t="inlineStr">
-        <is>
-          <t>Prep sauces: hollandaise, pesto, hummus</t>
+      <c r="B24" s="35" t="inlineStr">
+        <is>
+          <t>Prep sauces: hollandaise (use pasteurized eggs; hold it at 135 °F or above, or time-mark it and toss it after 4 hours), pesto, hummus</t>
         </is>
       </c>
       <c r="C24" s="29" t="inlineStr">
@@ -1641,9 +1641,9 @@
       <c r="A35" s="27" t="n">
         <v>26</v>
       </c>
-      <c r="B35" s="28" t="inlineStr">
-        <is>
-          <t>Sanitize work surfaces</t>
+      <c r="B35" s="36" t="inlineStr">
+        <is>
+          <t>Sanitize work surfaces with an approved sanitizer at the label concentration: check it with a test strip</t>
         </is>
       </c>
       <c r="C35" s="29" t="inlineStr">
@@ -1853,7 +1853,7 @@
     <row r="5">
       <c r="A5" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">  DINING ROOM</t>
+          <t xml:space="preserve">  SEATING AREA</t>
         </is>
       </c>
       <c r="B5" s="26" t="n"/>
@@ -2177,9 +2177,9 @@
       <c r="A18" s="27" t="n">
         <v>12</v>
       </c>
-      <c r="B18" s="28" t="inlineStr">
-        <is>
-          <t>Check that ashtrays are clean (smoking area)</t>
+      <c r="B18" s="36" t="inlineStr">
+        <is>
+          <t>Check that ashtrays are clean (only if local law allows smoking on your patio)</t>
         </is>
       </c>
       <c r="C18" s="29" t="inlineStr">
@@ -2752,9 +2752,9 @@
       <c r="A9" s="31" t="n">
         <v>4</v>
       </c>
-      <c r="B9" s="32" t="inlineStr">
-        <is>
-          <t>Check the machine pressure (9 bar)</t>
+      <c r="B9" s="35" t="inlineStr">
+        <is>
+          <t>Check the brew pressure gauge during the test shot (about 9 bar)</t>
         </is>
       </c>
       <c r="C9" s="29" t="inlineStr">
@@ -3156,9 +3156,9 @@
       <c r="A25" s="31" t="n">
         <v>18</v>
       </c>
-      <c r="B25" s="32" t="inlineStr">
-        <is>
-          <t>Brew the day's drip / batch brew</t>
+      <c r="B25" s="35" t="inlineStr">
+        <is>
+          <t>Brew the day's drip / batch brew; if you serve cold brew, filter the batch that finished steeping and store it covered at 41 °F or below, date-marked (7 days max counting the brew day)</t>
         </is>
       </c>
       <c r="C25" s="29" t="inlineStr">
@@ -3785,9 +3785,9 @@
       <c r="A14" s="27" t="n">
         <v>8</v>
       </c>
-      <c r="B14" s="28" t="inlineStr">
-        <is>
-          <t>Clean work surfaces and cutting boards</t>
+      <c r="B14" s="36" t="inlineStr">
+        <is>
+          <t>Clean and sanitize work surfaces and cutting boards; check the sanitizer with a test strip (range on its label)</t>
         </is>
       </c>
       <c r="C14" s="29" t="inlineStr">
@@ -3962,7 +3962,7 @@
       </c>
       <c r="B21" s="32" t="inlineStr">
         <is>
-          <t>Check that the walk-ins are closed and at temperature (cooler 41 °F or below, freezer 0 °F or below) — log reading: ____ °F</t>
+          <t>Check that the coolers and freezer are closed and at temperature (cooler 41 °F or below, freezer 0 °F or below) — log reading: cooler ____ °F · freezer ____ °F</t>
         </is>
       </c>
       <c r="C21" s="29" t="inlineStr">
@@ -4319,7 +4319,7 @@
     <row r="5">
       <c r="A5" s="25" t="inlineStr">
         <is>
-          <t xml:space="preserve">  DINING ROOM &amp; FURNITURE</t>
+          <t xml:space="preserve">  SEATING AREA &amp; FURNITURE</t>
         </is>
       </c>
       <c r="B5" s="26" t="n"/>
@@ -4335,7 +4335,7 @@
       </c>
       <c r="B6" s="28" t="inlineStr">
         <is>
-          <t>Break down tables: collect tablecloths, silverware, glasses</t>
+          <t>Break down tables: collect placemats/napkins, silverware, glasses</t>
         </is>
       </c>
       <c r="C6" s="29" t="inlineStr">
@@ -4562,9 +4562,9 @@
       <c r="A15" s="31" t="n">
         <v>9</v>
       </c>
-      <c r="B15" s="32" t="inlineStr">
-        <is>
-          <t>Collect and empty the ashtrays</t>
+      <c r="B15" s="35" t="inlineStr">
+        <is>
+          <t>Collect and empty the ashtrays (if you have a smoking area)</t>
         </is>
       </c>
       <c r="C15" s="29" t="inlineStr">
@@ -5110,9 +5110,9 @@
       <c r="A7" s="31" t="n">
         <v>2</v>
       </c>
-      <c r="B7" s="32" t="inlineStr">
-        <is>
-          <t>Clean the portafilters with hot water</t>
+      <c r="B7" s="35" t="inlineStr">
+        <is>
+          <t>Soak the portafilters and baskets in espresso machine cleaner (per its label), then rinse with hot water</t>
         </is>
       </c>
       <c r="C7" s="29" t="inlineStr">
@@ -5339,9 +5339,9 @@
       <c r="A16" s="27" t="n">
         <v>10</v>
       </c>
-      <c r="B16" s="28" t="inlineStr">
-        <is>
-          <t>Empty and clean the drip coffee airpots</t>
+      <c r="B16" s="36" t="inlineStr">
+        <is>
+          <t>Empty and clean the drip coffee airpots; if you serve cold brew, start tomorrow's batch in a clean, covered container, steeped in the cooler unless your health department allows room-temperature steeping</t>
         </is>
       </c>
       <c r="C16" s="29" t="inlineStr">
@@ -5435,7 +5435,7 @@
       </c>
       <c r="B20" s="36" t="inlineStr">
         <is>
-          <t>Put opened milk (and cold brew, if you serve it) in the walk-in cooler at 41 °F or below, covered and dated; the date on the label rules</t>
+          <t>Put opened milk (and cold brew, if you serve it) in the cooler at 41 °F or below, covered and date-marked: 7 days max counting the day it was opened, never past the use-by date on the label</t>
         </is>
       </c>
       <c r="C20" s="29" t="inlineStr">
@@ -5527,9 +5527,9 @@
       <c r="A24" s="27" t="n">
         <v>16</v>
       </c>
-      <c r="B24" s="28" t="inlineStr">
-        <is>
-          <t>Clean and sanitize the bar top</t>
+      <c r="B24" s="36" t="inlineStr">
+        <is>
+          <t>Clean and sanitize the bar top; check the sanitizer with a test strip (range on its label)</t>
         </is>
       </c>
       <c r="C24" s="29" t="inlineStr">
@@ -5610,7 +5610,7 @@
       </c>
       <c r="B27" s="32" t="inlineStr">
         <is>
-          <t>Empty the ice bin</t>
+          <t>Empty, clean and sanitize the ice bin</t>
         </is>
       </c>
       <c r="C27" s="29" t="inlineStr">

</xml_diff>